<commit_message>
Update Tools and Translations
</commit_message>
<xml_diff>
--- a/Docs/Translation FHM Table.xlsx
+++ b/Docs/Translation FHM Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Games\Emulator\ACI-Reverse-Engineering\ACI-Localization-Research\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11049BCC-EF71-49C0-A4C3-CE83613C89A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA412AB6-DFBE-410E-B60B-A504DBB14874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5940" yWindow="2130" windowWidth="28800" windowHeight="15375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3150" yWindow="3915" windowWidth="33510" windowHeight="15375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
   <si>
     <t>FHM HashID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -124,19 +124,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MenuHeader_*_*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>InfoHeader_*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Movie Font</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MsnNameLocal_*</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -197,10 +185,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PartsSName_*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Movie Font
 A_OTF_Shin_Go_Pr5_R30_radio</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -216,28 +200,78 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MsnDateDesc_micp*
+    <t>UI Localization 1
+UI Localization 2
+MenuHeader_*_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 1
+MsnNameLocal_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 1
+MsnDateDesc_micp*
 MsnDateDesc_miff*
 MsnLocationDesc_micp*</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>InfoItem_AcStat_*
+    <t>UI Localization 1
+TabHeader_Rslt_*
+InfoItem_RsltScoreDetail_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 1
+AcName_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 1
+MsnName_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 1
+UI Localization 2
+InfoHeader_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 2
+PartsSName_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 2
+AcTypeName_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 2
+MenuItem_Title_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 2
+InfoItem_AcStat_*
 InfoItem_PartsSlot_*
 InfoItem_WpnStat_*
-InfoItem_WpnDetail_*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AcTypeName_*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AcName_*</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MsnName_*</t>
+InfoItem_WpnDetail_*
+InfoItem_Title_*</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x0ac159b1</t>
+  </si>
+  <si>
+    <t>0 - 0.act</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Localization 1 Ingame</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -991,6 +1025,172 @@
         <a:xfrm>
           <a:off x="14763751" y="6389078"/>
           <a:ext cx="1648558" cy="621742"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1800419" cy="446942"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="图片 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E08DCB1E-CC9A-408A-AF7D-1C6937BB9818}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5912827" y="2036885"/>
+          <a:ext cx="1800419" cy="446942"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>29308</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>468923</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2403231" cy="402795"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="图片 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92273F5A-B14A-40C1-9667-9B8094EBCB0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5942135" y="2505808"/>
+          <a:ext cx="2403231" cy="402795"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1362809</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>478083</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="图片 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B72D10D-8F95-1FFB-EAA0-51DFAD4AD080}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5912828" y="2036886"/>
+          <a:ext cx="1362808" cy="478082"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>21981</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>293077</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>4176346</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>642873</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="图片 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32243FC4-A78B-76A9-BB30-86428FBB801C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5934808" y="7297615"/>
+          <a:ext cx="4154365" cy="349796"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1265,7 +1465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="29" customWidth="1"/>
@@ -1284,7 +1484,7 @@
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1326,7 +1526,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -1351,10 +1551,10 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1365,10 +1565,10 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1382,7 +1582,7 @@
         <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -1421,10 +1621,24 @@
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1440,11 +1654,12 @@
   <cols>
     <col min="1" max="1" width="29.75" customWidth="1"/>
     <col min="2" max="2" width="47.875" customWidth="1"/>
-    <col min="3" max="3" width="43.625" customWidth="1"/>
+    <col min="3" max="3" width="83.5" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="25.25" customWidth="1"/>
     <col min="6" max="6" width="22.25" customWidth="1"/>
     <col min="7" max="7" width="24.375" customWidth="1"/>
+    <col min="8" max="8" width="20.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -1457,69 +1672,75 @@
     </row>
     <row r="2" spans="1:7" ht="87.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="120" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="96.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="139.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update .uifont drag in
</commit_message>
<xml_diff>
--- a/Docs/Translation FHM Table.xlsx
+++ b/Docs/Translation FHM Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Games\Emulator\ACI-Reverse-Engineering\ACI-Localization-Research\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA412AB6-DFBE-410E-B60B-A504DBB14874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FFAEB5-6743-4B6B-8650-A7B58A1088CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3150" yWindow="3915" windowWidth="33510" windowHeight="15375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3150" yWindow="3915" windowWidth="35250" windowHeight="15375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="55">
   <si>
     <t>FHM HashID</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -149,11 +149,6 @@
   </si>
   <si>
     <t>Credit Font</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>UI Font 1
-Futura_MdCn_BT26</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -192,11 +187,6 @@
   <si>
     <t>Campaign 1 Font
 A_OTF_Shin_Go_Pr5_R20_radio</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>UI Font 2
-Futura_MdCn_BT26</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -272,6 +262,12 @@
   </si>
   <si>
     <t>UI Localization 1 Ingame</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI Font 1
+UI Font 2
+Futura_MdCn_BT26</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -536,13 +532,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>2716106</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>1260231</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -595,15 +591,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>1221987</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>490304</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -861,13 +857,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>3248823</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>395654</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1037,7 +1033,7 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1800419" cy="446942"/>
@@ -1076,8 +1072,8 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>29308</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>468923</xdr:rowOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2403231" cy="402795"/>
     <xdr:pic>
@@ -1113,15 +1109,15 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>1</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>1362809</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>478083</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1537,10 +1533,10 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -1551,10 +1547,10 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1624,7 +1620,7 @@
         <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1632,13 +1628,13 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" t="s">
         <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1654,7 +1650,7 @@
   <cols>
     <col min="1" max="1" width="29.75" customWidth="1"/>
     <col min="2" max="2" width="47.875" customWidth="1"/>
-    <col min="3" max="3" width="83.5" customWidth="1"/>
+    <col min="3" max="3" width="55.25" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="25.25" customWidth="1"/>
     <col min="6" max="6" width="22.25" customWidth="1"/>
@@ -1672,75 +1668,73 @@
     </row>
     <row r="2" spans="1:7" ht="87.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="1" t="s">
+    </row>
+    <row r="4" spans="1:7" ht="58.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="135.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="139.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="F8" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>